<commit_message>
updated on sep 21
</commit_message>
<xml_diff>
--- a/1234567 (1).xlsx
+++ b/1234567 (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ACER\Desktop\python\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C415888B-8742-4A5D-95D2-EFDD4FD13FE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BACB147C-AAB0-4054-A041-F9CE7D052489}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="68">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -2170,26 +2170,50 @@
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A31" s="13"/>
-      <c r="B31" s="14"/>
-      <c r="C31" s="14"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
-      <c r="F31" s="14"/>
-      <c r="G31" s="14"/>
-      <c r="H31" s="14"/>
-      <c r="I31" s="15" t="str">
+      <c r="A31" s="13">
+        <v>46287</v>
+      </c>
+      <c r="B31" s="14">
+        <v>600</v>
+      </c>
+      <c r="C31" s="14">
+        <v>30</v>
+      </c>
+      <c r="D31" s="14">
+        <v>40</v>
+      </c>
+      <c r="E31" s="14">
+        <v>20</v>
+      </c>
+      <c r="F31" s="14">
+        <v>250</v>
+      </c>
+      <c r="G31" s="14">
+        <v>5</v>
+      </c>
+      <c r="H31" s="14">
+        <v>10</v>
+      </c>
+      <c r="I31" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J31" s="15" t="str">
+        <v>950</v>
+      </c>
+      <c r="J31" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K31" s="16"/>
-      <c r="L31" s="16"/>
-      <c r="M31" s="16"/>
-      <c r="N31" s="17"/>
+        <v>490</v>
+      </c>
+      <c r="K31" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L31" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M31" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="N31" s="17" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A32" s="13"/>

</xml_diff>